<commit_message>
Switch CZ/SK CM shortlist to league-based filtering
export_cz_sk_young_cms.py now filters by which Czech/Slovak league file
the player is in (Czech, Czech II, Czech U17, Czech U19, Slovakia,
Slovakia II) instead of passport nationality, matching the treatment
already applied to screen_six_eight.py. Candidate count rises from 156
to 193, now including foreign nationals playing in these leagues (e.g.
A. Zeljković/Slovenia at Viktoria Plzeň, C. Zafeiris/Greece at Slavia
Praha) instead of only CZ/SK passport holders, some of whom played
abroad (L. Ambros in Poland, K. Daněk in Austria — now excluded since
they don't play in a CZ/SK league).

Regenerated CZ_SK_Young_CMs_Lamberts.xlsx from the updated shortlist.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wzh48iso9dywMF7h3c4ehR
</commit_message>
<xml_diff>
--- a/data/CZ_SK_Young_CMs_Lamberts.xlsx
+++ b/data/CZ_SK_Young_CMs_Lamberts.xlsx
@@ -84,12 +84,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00626567"/>
+        <fgColor rgb="00117A65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00117A65"/>
+        <fgColor rgb="00626567"/>
       </patternFill>
     </fill>
     <fill>
@@ -147,10 +147,10 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T10"/>
+  <dimension ref="A1:T12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -540,7 +540,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Jamestown / Marc Lamberts methodology  ·  Top 7 of 7 scored (real market value only, 156 candidates total)  ·  Ranked by Lamberts Index (SQS Rank − Market Value Rank)</t>
+          <t>Jamestown / Marc Lamberts methodology  ·  Top 9 of 9 scored (real market value only, 193 candidates total)  ·  Ranked by Lamberts Index (SQS Rank − Market Value Rank)</t>
         </is>
       </c>
     </row>
@@ -649,25 +649,25 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>L. Ambros</t>
+          <t>M. Breznik</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Górnik Zabrze</t>
+          <t>Malženice</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Slovakia II</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>1968</v>
+        <v>1828</v>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
@@ -684,10 +684,10 @@
         </is>
       </c>
       <c r="I4" s="4" t="n">
-        <v>85.45999999999999</v>
+        <v>91.14</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>50.59</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
@@ -695,49 +695,49 @@
         </is>
       </c>
       <c r="L4" s="4" t="n">
-        <v>250000</v>
+        <v>150000</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>427300</v>
+        <v>273420</v>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>1.7×</t>
+          <t>1.8×</t>
         </is>
       </c>
       <c r="O4" s="4" t="n">
-        <v>31.8</v>
+        <v>37.4</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>0.09</v>
+        <v>0.15</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>4.85</v>
+        <v>7.73</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>0.46</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>P. Kulíšek</t>
+          <t>K. Palumets</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Hanácká</t>
+          <t>Podbrezová</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Czech II</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
@@ -745,72 +745,72 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
-        <v>1622</v>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>FAIR VALUE</t>
+        <v>2154</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>ELITE VALUE</t>
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>11.85</v>
-      </c>
-      <c r="J5" s="9" t="n">
-        <v>9.380000000000001</v>
-      </c>
-      <c r="K5" s="10" t="inlineStr">
-        <is>
-          <t>DEPTH</t>
+        <v>87.64</v>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>61.06</v>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>CLEAR UPGRADE</t>
         </is>
       </c>
       <c r="L5" s="7" t="n">
-        <v>50000</v>
+        <v>200000</v>
       </c>
       <c r="M5" s="7" t="n">
-        <v>11850</v>
+        <v>350560</v>
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>0.2×</t>
+          <t>1.8×</t>
         </is>
       </c>
       <c r="O5" s="7" t="n">
-        <v>-41.9</v>
+        <v>33.9</v>
       </c>
       <c r="P5" s="7" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="Q5" s="7" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="R5" s="7" t="n">
-        <v>0.02</v>
+        <v>0.12</v>
       </c>
       <c r="S5" s="7" t="n">
-        <v>5.55</v>
+        <v>6.89</v>
       </c>
       <c r="T5" s="7" t="n">
-        <v>0.06</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>S. Grygar</t>
+          <t>E. Metu</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Ružomberok</t>
+          <t>FC Košice</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -819,33 +819,33 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>2065</v>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>FAIR VALUE</t>
+        <v>598</v>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>VALUE</t>
         </is>
       </c>
       <c r="I6" s="4" t="n">
-        <v>31.36</v>
+        <v>35.79</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>9.16</v>
-      </c>
-      <c r="K6" s="10" t="inlineStr">
+        <v>13.59</v>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>DEPTH</t>
         </is>
@@ -854,46 +854,46 @@
         <v>175000</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>109760</v>
+        <v>125265</v>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>0.6×</t>
+          <t>0.7×</t>
         </is>
       </c>
       <c r="O6" s="4" t="n">
-        <v>-22.3</v>
+        <v>-17.9</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>6.19</v>
+        <v>5.12</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>M. Šviderský</t>
+          <t>P. Kulíšek</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Slovácko</t>
+          <t>Hanácká</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Czech</t>
+          <t>Czech II</t>
         </is>
       </c>
       <c r="D7" s="7" t="n">
@@ -901,46 +901,46 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>1219</v>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>OVERPRICED</t>
+        <v>1622</v>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>FAIR VALUE</t>
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>33.18</v>
-      </c>
-      <c r="J7" s="9" t="n">
-        <v>-9.67</v>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
+        <v>11.85</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
         <is>
           <t>DEPTH</t>
         </is>
       </c>
       <c r="L7" s="7" t="n">
-        <v>300000</v>
+        <v>50000</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>199080</v>
+        <v>11850</v>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>0.7×</t>
+          <t>0.2×</t>
         </is>
       </c>
       <c r="O7" s="7" t="n">
-        <v>-20.5</v>
+        <v>-41.9</v>
       </c>
       <c r="P7" s="7" t="n">
         <v>0</v>
@@ -949,33 +949,33 @@
         <v>0</v>
       </c>
       <c r="R7" s="7" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="S7" s="7" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="T7" s="7" t="n">
         <v>0.06</v>
-      </c>
-      <c r="S7" s="7" t="n">
-        <v>5.32</v>
-      </c>
-      <c r="T7" s="7" t="n">
-        <v>0.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>K. Daněk</t>
+          <t>S. Grygar</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>LASK</t>
+          <t>Ružomberok</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
@@ -984,67 +984,67 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>1485</v>
-      </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>OVERPRICED</t>
+        <v>2065</v>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>FAIR VALUE</t>
         </is>
       </c>
       <c r="I8" s="4" t="n">
-        <v>65.75</v>
+        <v>31.36</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>-12</v>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>CLEAR UPGRADE</t>
+        <v>9.16</v>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>DEPTH</t>
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>1000000</v>
+        <v>175000</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>1315000</v>
+        <v>109760</v>
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>1.3×</t>
+          <t>0.6×</t>
         </is>
       </c>
       <c r="O8" s="4" t="n">
-        <v>12</v>
+        <v>-22.3</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>0.16</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>3.58</v>
+        <v>6.19</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>0.67</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>M. Náprstek</t>
+          <t>A. Zeljković</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Teplice</t>
+          <t>Viktoria Plzeň</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -1053,85 +1053,85 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>1292</v>
-      </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>OVERPRICED</t>
+        <v>466</v>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>FAIR VALUE</t>
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>4.11</v>
-      </c>
-      <c r="J9" s="9" t="n">
-        <v>-34.46</v>
-      </c>
-      <c r="K9" s="10" t="inlineStr">
-        <is>
-          <t>DEPTH</t>
+        <v>92.04000000000001</v>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>CLEAR UPGRADE</t>
         </is>
       </c>
       <c r="L9" s="7" t="n">
-        <v>275000</v>
+        <v>2000000</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>27500</v>
+        <v>3681600</v>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>0.1×</t>
+          <t>1.8×</t>
         </is>
       </c>
       <c r="O9" s="7" t="n">
-        <v>-49.6</v>
+        <v>38.3</v>
       </c>
       <c r="P9" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="7" t="n">
-        <v>0</v>
+        <v>0.19</v>
       </c>
       <c r="R9" s="7" t="n">
         <v>0.06</v>
       </c>
       <c r="S9" s="7" t="n">
-        <v>3.97</v>
+        <v>6.76</v>
       </c>
       <c r="T9" s="7" t="n">
-        <v>0.14</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>M. Sauer</t>
+          <t>M. Šviderský</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Slovácko</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Czech</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
@@ -1140,11 +1140,11 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>807</v>
+        <v>1219</v>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
@@ -1152,44 +1152,200 @@
         </is>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5.58</v>
+        <v>33.18</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>-75.15000000000001</v>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
+        <v>-9.67</v>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
         <is>
           <t>DEPTH</t>
         </is>
       </c>
       <c r="L10" s="4" t="n">
-        <v>1300000</v>
+        <v>300000</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>145080</v>
+        <v>199080</v>
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>0.1×</t>
+          <t>0.7×</t>
         </is>
       </c>
       <c r="O10" s="4" t="n">
-        <v>-48.1</v>
+        <v>-20.5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>0.01</v>
+        <v>0.06</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3.9</v>
+        <v>5.32</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>0.11</v>
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>C. Zafeiris</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Slavia Praha</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Czech</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Greece, Norway</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>1230</v>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>OVERPRICED</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>73.06999999999999</v>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>-21.91</v>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>CLEAR UPGRADE</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>10229800</v>
+      </c>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>1.5×</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="P11" s="7" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Q11" s="7" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="R11" s="7" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="S11" s="7" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="T11" s="7" t="n">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>M. Náprstek</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Teplice</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Czech</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>1292</v>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>OVERPRICED</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>-34.46</v>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>DEPTH</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>275000</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>27500</v>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>0.1×</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>-49.6</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <v>0.14</v>
       </c>
     </row>
   </sheetData>
@@ -1223,7 +1379,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Modeled on Matthew Benham / Brentford's data-led approach  ·  Top 15 of 156  ·  weights underlying chance creation (xA, key passes, xG, progressive passing)  ·  proxy score, not the club's proprietary formula</t>
+          <t>Modeled on Matthew Benham / Brentford's data-led approach  ·  Top 15 of 193  ·  weights underlying chance creation (xA, key passes, xG, progressive passing)  ·  proxy score, not the club's proprietary formula</t>
         </is>
       </c>
     </row>
@@ -1705,29 +1861,29 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Š. Sedlák</t>
+          <t>D. Teah</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Vysočina Jihlava U19</t>
+          <t>Slavia Praha</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Czech U19</t>
+          <t>Czech II</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Liberia</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>615</v>
+        <v>727</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
@@ -1735,50 +1891,50 @@
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>93.34</v>
+        <v>94.63</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>0.17</v>
+        <v>0.11</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0.59</v>
+        <v>0.74</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>0.2</v>
+        <v>0.11</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>5.41</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>A. Gajdoš</t>
+          <t>Š. Sedlák</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Slovan Bratislava</t>
+          <t>Vysočina Jihlava U19</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Czech U19</t>
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1417</v>
+        <v>615</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -1786,50 +1942,50 @@
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>92.77</v>
+        <v>93.34</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>0.17</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.38</v>
+        <v>0.59</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>0.2</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>6.8</v>
+        <v>5.41</v>
       </c>
       <c r="M13" s="7" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>D. Kolar</t>
+          <t>A. Gajdoš</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>České Budějovice U17</t>
+          <t>Slovan Bratislava</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Czech U17</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>795</v>
+        <v>1417</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -1837,33 +1993,33 @@
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>92.62</v>
+        <v>92.77</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>0.11</v>
+        <v>0.17</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0.45</v>
+        <v>0.38</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>0.14</v>
+        <v>0.2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>8.83</v>
+        <v>6.8</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>0.23</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>L. Havrlík</t>
+          <t>D. Kolar</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Sparta Praha U17</t>
+          <t>České Budějovice U17</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -1880,7 +2036,7 @@
         </is>
       </c>
       <c r="F15" s="7" t="n">
-        <v>424</v>
+        <v>795</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
@@ -1888,42 +2044,42 @@
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>92.25</v>
+        <v>92.62</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.29</v>
+        <v>0.11</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.42</v>
+        <v>0.45</v>
       </c>
       <c r="K15" s="7" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="M15" s="7" t="n">
         <v>0.23</v>
-      </c>
-      <c r="L15" s="7" t="n">
-        <v>7.85</v>
-      </c>
-      <c r="M15" s="7" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>M. Brázda</t>
+          <t>L. Havrlík</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Zlín U19</t>
+          <t>Sparta Praha U17</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Czech U19</t>
+          <t>Czech U17</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
@@ -1931,7 +2087,7 @@
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>1255</v>
+        <v>424</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
@@ -1939,19 +2095,19 @@
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>92.15000000000001</v>
+        <v>92.25</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>0.19</v>
+        <v>0.29</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>0.27</v>
+        <v>0.23</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>8.529999999999999</v>
+        <v>7.85</v>
       </c>
       <c r="M16" s="4" t="n">
         <v>0</v>
@@ -1960,12 +2116,12 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>A. Tichánek</t>
+          <t>M. Brázda</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Vysočina Jihlava U19</t>
+          <t>Zlín U19</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -1974,7 +2130,7 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
@@ -1982,7 +2138,7 @@
         </is>
       </c>
       <c r="F17" s="7" t="n">
-        <v>882</v>
+        <v>1255</v>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
@@ -1990,38 +2146,38 @@
         </is>
       </c>
       <c r="H17" s="7" t="n">
-        <v>91.14</v>
+        <v>92.15000000000001</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.31</v>
+        <v>0.43</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>0.17</v>
+        <v>0.27</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>5.82</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="M17" s="7" t="n">
-        <v>0.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>J. Zadrobílek</t>
+          <t>A. Tichánek</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Sparta Praha U19</t>
+          <t>Vysočina Jihlava U19</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Czech U17</t>
+          <t>Czech U19</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">
@@ -2033,7 +2189,7 @@
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>1063</v>
+        <v>882</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
@@ -2041,22 +2197,22 @@
         </is>
       </c>
       <c r="H18" s="4" t="n">
-        <v>90.98999999999999</v>
+        <v>91.14</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>0.13</v>
+        <v>0.21</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>0.51</v>
+        <v>0.31</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>0.58</v>
+        <v>0.17</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>7.87</v>
+        <v>5.82</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>0</v>
+        <v>0.31</v>
       </c>
     </row>
   </sheetData>
@@ -2090,7 +2246,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Modeled on the Red Bull Group pipeline archetype  ·  Top 15 of 156  ·  weights youth, pressing/duel intensity and progressive ball-carrying  ·  proxy score, not the club's proprietary formula</t>
+          <t>Modeled on the Red Bull Group pipeline archetype  ·  Top 15 of 193  ·  weights youth, pressing/duel intensity and progressive ball-carrying  ·  proxy score, not the club's proprietary formula</t>
         </is>
       </c>
     </row>
@@ -2493,29 +2649,29 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>J. Base</t>
+          <t>F. Bzdyl</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>FC Hradec Králové U17</t>
+          <t>Žilina</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Czech U17</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1277</v>
+        <v>1047</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
@@ -2523,22 +2679,22 @@
         </is>
       </c>
       <c r="H10" s="4" t="n">
-        <v>99.79000000000001</v>
+        <v>99.84</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1.9</v>
+        <v>1.72</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>69.62</v>
+        <v>72.31</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2.89</v>
+        <v>2.66</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3.45</v>
+        <v>3.27</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>53.06</v>
+        <v>63.16</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>57.89</v>
@@ -2547,12 +2703,12 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>S. Mladen</t>
+          <t>J. Base</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Dukla Praha U17</t>
+          <t>FC Hradec Králové U17</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -2561,7 +2717,7 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
@@ -2569,7 +2725,7 @@
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>994</v>
+        <v>1277</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
@@ -2577,53 +2733,53 @@
         </is>
       </c>
       <c r="H11" s="7" t="n">
-        <v>99.76000000000001</v>
+        <v>99.79000000000001</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>3.17</v>
+        <v>1.9</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>68.89</v>
+        <v>69.62</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>3.17</v>
+        <v>2.89</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>6.88</v>
+        <v>3.45</v>
       </c>
       <c r="M11" s="7" t="n">
-        <v>51.32</v>
+        <v>53.06</v>
       </c>
       <c r="N11" s="7" t="n">
-        <v>32.26</v>
+        <v>57.89</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>R. Filip</t>
+          <t>S. Mladen</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Baník Ostrava U19</t>
+          <t>Dukla Praha U17</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Czech U19</t>
+          <t>Czech U17</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>742</v>
+        <v>994</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
@@ -2631,25 +2787,25 @@
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>99.69</v>
+        <v>99.76000000000001</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>1.94</v>
+        <v>3.17</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>73.33</v>
+        <v>68.89</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4.37</v>
+        <v>3.17</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>1.33</v>
+        <v>6.88</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>63.64</v>
+        <v>51.32</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>36.36</v>
+        <v>32.26</v>
       </c>
     </row>
     <row r="13">
@@ -2707,12 +2863,12 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>J. Zima</t>
+          <t>R. Filip</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Pardubice U19</t>
+          <t>Baník Ostrava U19</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -2721,15 +2877,15 @@
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>788</v>
+        <v>742</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -2737,45 +2893,45 @@
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>99.61</v>
+        <v>99.69</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>1.71</v>
+        <v>1.94</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>60</v>
+        <v>73.33</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3.88</v>
+        <v>4.37</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2.86</v>
+        <v>1.33</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>72</v>
+        <v>63.64</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>66.67</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>F. Rada</t>
+          <t>J. Zima</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Viktoria Plzeň U17</t>
+          <t>Pardubice U19</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Czech U17</t>
+          <t>Czech U19</t>
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
@@ -2783,7 +2939,7 @@
         </is>
       </c>
       <c r="F15" s="7" t="n">
-        <v>719</v>
+        <v>788</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
@@ -2791,45 +2947,45 @@
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>99.58</v>
+        <v>99.61</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>1.13</v>
+        <v>1.71</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>74.70999999999999</v>
+        <v>60</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>4.13</v>
+        <v>3.88</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>1.75</v>
+        <v>2.86</v>
       </c>
       <c r="M15" s="7" t="n">
-        <v>64.29000000000001</v>
+        <v>72</v>
       </c>
       <c r="N15" s="7" t="n">
-        <v>56.25</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>D. Ledvinka</t>
+          <t>F. Rada</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Dukla Praha U19</t>
+          <t>Viktoria Plzeň U17</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Czech U19</t>
+          <t>Czech U17</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
@@ -2837,7 +2993,7 @@
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>528</v>
+        <v>719</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
@@ -2845,45 +3001,45 @@
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>99.56999999999999</v>
+        <v>99.58</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>2.05</v>
+        <v>1.13</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>62.16</v>
+        <v>74.70999999999999</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>3.92</v>
+        <v>4.13</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>3.92</v>
+        <v>1.75</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>43.48</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>75</v>
+        <v>56.25</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>R. Horák</t>
+          <t>D. Ledvinka</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Slovácko</t>
+          <t>Dukla Praha U19</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Czech II</t>
+          <t>Czech U19</t>
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
@@ -2891,7 +3047,7 @@
         </is>
       </c>
       <c r="F17" s="7" t="n">
-        <v>1140</v>
+        <v>528</v>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
@@ -2899,45 +3055,45 @@
         </is>
       </c>
       <c r="H17" s="7" t="n">
-        <v>99.52</v>
+        <v>99.56999999999999</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>1.58</v>
+        <v>2.05</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>68.48</v>
+        <v>62.16</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>4.97</v>
+        <v>3.92</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>1.97</v>
+        <v>3.92</v>
       </c>
       <c r="M17" s="7" t="n">
-        <v>64</v>
+        <v>43.48</v>
       </c>
       <c r="N17" s="7" t="n">
-        <v>52.94</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>P. Filippov</t>
+          <t>R. Horák</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Podbrezová</t>
+          <t>Slovácko</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Czech U19</t>
+          <t>Czech II</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
@@ -2945,7 +3101,7 @@
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>776</v>
+        <v>1140</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
@@ -2953,25 +3109,25 @@
         </is>
       </c>
       <c r="H18" s="4" t="n">
-        <v>99.45999999999999</v>
+        <v>99.52</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>2.44</v>
+        <v>1.58</v>
       </c>
       <c r="J18" s="4" t="n">
+        <v>68.48</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="M18" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="K18" s="4" t="n">
-        <v>2.78</v>
-      </c>
-      <c r="L18" s="4" t="n">
-        <v>3.36</v>
-      </c>
-      <c r="M18" s="4" t="n">
-        <v>58.62</v>
-      </c>
       <c r="N18" s="4" t="n">
-        <v>50</v>
+        <v>52.94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>